<commit_message>
Fix Excel: clickable URLs in separate columns, rename to Module, remove S.No
https://claude.ai/code/session_018v8twwNDLhKYK2n2HVYhb1
</commit_message>
<xml_diff>
--- a/Substation_Workflow_Module_Guide.xlsx
+++ b/Substation_Workflow_Module_Guide.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Substation Workflows" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Substation Workflows'!$A$1:$C$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Substation Workflows'!$A$1:$D$123</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -36,6 +36,7 @@
     </font>
     <font>
       <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="2">
@@ -443,18 +444,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:D123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Workflow Name</t>
+          <t>Module</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -464,11 +466,16 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Source URLs</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="48" customHeight="1">
+          <t>Source URL 1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Source URL 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bid Process in Substation EPC Projects</t>
@@ -481,12 +488,16 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>1. https://constructionfront.com/epc-contract/
-2. https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="48" customHeight="1">
+          <t>https://constructionfront.com/epc-contract/</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1">
       <c r="A3" s="3" t="inlineStr"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
@@ -495,12 +506,16 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.procore.com/library/epc-contractors
-2. https://prismecs.com/blog/understanding-the-lifecycle-of-epc-solutions-services</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="48" customHeight="1">
+          <t>https://www.procore.com/library/epc-contractors</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>https://prismecs.com/blog/understanding-the-lifecycle-of-epc-solutions-services</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
       <c r="A4" s="3" t="inlineStr"/>
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -509,12 +524,16 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.euci.com/event_post/epc-contracts/
-2. https://dancumberlandlabs.com/blog/epc-engineering-procurement-construction/</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="48" customHeight="1">
+          <t>https://www.euci.com/event_post/epc-contracts/</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>https://dancumberlandlabs.com/blog/epc-engineering-procurement-construction/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
       <c r="A5" s="3" t="inlineStr"/>
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -523,12 +542,16 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-design-engineering
-2. https://keentelengineering.com/a-guide-to-the-substation-design-process</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-design-engineering</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>https://keentelengineering.com/a-guide-to-the-substation-design-process</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
       <c r="A6" s="3" t="inlineStr"/>
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -537,12 +560,16 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>1. https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents
-2. https://electrical-engineering-portal.com/checks-for-successful-substation-factory-acceptance-testing</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
+          <t>https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical-engineering-portal.com/checks-for-successful-substation-factory-acceptance-testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
       <c r="A7" s="3" t="inlineStr"/>
       <c r="B7" s="3" t="inlineStr">
         <is>
@@ -551,12 +578,16 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>1. https://rkstrainings.com/what-is-project-management-in-epc/
-2. https://prismecs.com/blog/understanding-the-lifecycle-of-epc-solutions-services</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1">
+          <t>https://rkstrainings.com/what-is-project-management-in-epc/</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>https://prismecs.com/blog/understanding-the-lifecycle-of-epc-solutions-services</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
       <c r="A8" s="3" t="inlineStr"/>
       <c r="B8" s="3" t="inlineStr">
         <is>
@@ -565,12 +596,16 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>1. https://rkstrainings.com/what-is-project-management-in-epc/
-2. https://www.pmi.org/learning/library/realizing-engineering-procurement-construction-projects-7173</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
+          <t>https://rkstrainings.com/what-is-project-management-in-epc/</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pmi.org/learning/library/realizing-engineering-procurement-construction-projects-7173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
       <c r="A9" s="3" t="inlineStr"/>
       <c r="B9" s="3" t="inlineStr">
         <is>
@@ -579,12 +614,16 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.mayerbrown.com/Files/Publication/35328234-d6f9-49c7-bbe8-964945bb9158/Presentation/PublicationAttachment/96527455-174f-4e1a-9a9c-9a1d66e9bde3/EPC_contracts_jan15_hosie.pdf
-2. https://www.pmi.org/learning/library/realizing-engineering-procurement-construction-projects-7173</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="48" customHeight="1">
+          <t>https://www.mayerbrown.com/Files/Publication/35328234-d6f9-49c7-bbe8-964945bb9158/Presentation/PublicationAttachment/96527455-174f-4e1a-9a9c-9a1d66e9bde3/EPC_contracts_jan15_hosie.pdf</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pmi.org/learning/library/realizing-engineering-procurement-construction-projects-7173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
       <c r="A10" s="3" t="inlineStr"/>
       <c r="B10" s="3" t="inlineStr">
         <is>
@@ -593,12 +632,16 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.euci.com/event_post/epc-contracts/
-2. https://www.pillsburylaw.com/a/web/157254/EPC-Agreement-Provisions.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="48" customHeight="1">
+          <t>https://www.euci.com/event_post/epc-contracts/</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pillsburylaw.com/a/web/157254/EPC-Agreement-Provisions.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
       <c r="A11" s="3" t="inlineStr"/>
       <c r="B11" s="3" t="inlineStr">
         <is>
@@ -607,12 +650,16 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.pillsburylaw.com/a/web/157254/EPC-Agreement-Provisions.pdf
-2. https://fidic.org/sites/default/files/The%20FIDIC%20Contracts%20Guide.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="48" customHeight="1">
+          <t>https://www.pillsburylaw.com/a/web/157254/EPC-Agreement-Provisions.pdf</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>https://fidic.org/sites/default/files/The%20FIDIC%20Contracts%20Guide.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
       <c r="A12" s="3" t="inlineStr"/>
       <c r="B12" s="3" t="inlineStr">
         <is>
@@ -621,12 +668,16 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.procore.com/library/epc-contractors
-2. https://www.sora.ro/2026/05/31/epc-versus-fidic-contracts/</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="48" customHeight="1">
+          <t>https://www.procore.com/library/epc-contractors</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sora.ro/2026/05/31/epc-versus-fidic-contracts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
       <c r="A13" s="3" t="inlineStr"/>
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -635,12 +686,16 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>1. https://relgrow.com/resources/dlp-full-form-in-construction/
-2. https://www.pillsburylaw.com/a/web/157254/EPC-Agreement-Provisions.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="48" customHeight="1">
+          <t>https://relgrow.com/resources/dlp-full-form-in-construction/</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pillsburylaw.com/a/web/157254/EPC-Agreement-Provisions.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
       <c r="A14" s="3" t="inlineStr"/>
       <c r="B14" s="3" t="inlineStr">
         <is>
@@ -649,12 +704,16 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>1. https://fidic.org/sites/default/files/The%20FIDIC%20Contracts%20Guide.pdf
-2. https://lauwtjunnji.weebly.com/uploads/1/0/1/7/10171621/fidic_-_conditions_of_contract_for_epc_(turnkey)_projects_(1999).pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="48" customHeight="1">
+          <t>https://fidic.org/sites/default/files/The%20FIDIC%20Contracts%20Guide.pdf</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>https://lauwtjunnji.weebly.com/uploads/1/0/1/7/10171621/fidic_-_conditions_of_contract_for_epc_(turnkey)_projects_(1999).pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Contract Finalization and Project Mobilization Process</t>
@@ -667,12 +726,16 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>1. https://pmri.in/epccompletion/
-2. https://relgrow.com/resources/dlp-full-form-in-construction/</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="48" customHeight="1">
+          <t>https://pmri.in/epccompletion/</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>https://relgrow.com/resources/dlp-full-form-in-construction/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
       <c r="A16" s="3" t="inlineStr"/>
       <c r="B16" s="3" t="inlineStr">
         <is>
@@ -681,12 +744,16 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>1. https://fidic.org/sites/default/files/The%20FIDIC%20Contracts%20Guide.pdf
-2. https://www.pillsburylaw.com/a/web/157254/EPC-Agreement-Provisions.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="48" customHeight="1">
+          <t>https://fidic.org/sites/default/files/The%20FIDIC%20Contracts%20Guide.pdf</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pillsburylaw.com/a/web/157254/EPC-Agreement-Provisions.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
       <c r="A17" s="3" t="inlineStr"/>
       <c r="B17" s="3" t="inlineStr">
         <is>
@@ -695,12 +762,16 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>1. https://petroedgeasia.net/training/engineering-procurement-construction-contracts-epc-training-course/
-2. https://fidic.org/sites/default/files/The%20FIDIC%20Contracts%20Guide.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="48" customHeight="1">
+          <t>https://petroedgeasia.net/training/engineering-procurement-construction-contracts-epc-training-course/</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>https://fidic.org/sites/default/files/The%20FIDIC%20Contracts%20Guide.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
       <c r="A18" s="3" t="inlineStr"/>
       <c r="B18" s="3" t="inlineStr">
         <is>
@@ -709,12 +780,16 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>1. https://fidic.org/sites/default/files/The%20FIDIC%20Contracts%20Guide.pdf
-2. https://constructionfront.com/epc-contract/</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="48" customHeight="1">
+          <t>https://fidic.org/sites/default/files/The%20FIDIC%20Contracts%20Guide.pdf</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>https://constructionfront.com/epc-contract/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
       <c r="A19" s="3" t="inlineStr"/>
       <c r="B19" s="3" t="inlineStr">
         <is>
@@ -723,12 +798,16 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>1. https://lauwtjunnji.weebly.com/uploads/1/0/1/7/10171621/fidic_-_conditions_of_contract_for_epc_(turnkey)_projects_(1999).pdf
-2. https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="48" customHeight="1">
+          <t>https://lauwtjunnji.weebly.com/uploads/1/0/1/7/10171621/fidic_-_conditions_of_contract_for_epc_(turnkey)_projects_(1999).pdf</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
       <c r="A20" s="3" t="inlineStr"/>
       <c r="B20" s="3" t="inlineStr">
         <is>
@@ -737,12 +816,16 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>1. https://pmri.in/epccompletion/
-2. https://rkstrainings.com/what-is-project-management-in-epc/</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="48" customHeight="1">
+          <t>https://pmri.in/epccompletion/</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>https://rkstrainings.com/what-is-project-management-in-epc/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
       <c r="A21" s="3" t="inlineStr"/>
       <c r="B21" s="3" t="inlineStr">
         <is>
@@ -751,12 +834,16 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>1. https://projectmanagement123.com/project-completion-and-handover-procedure/
-2. https://pmri.in/epccompletion/</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="48" customHeight="1">
+          <t>https://projectmanagement123.com/project-completion-and-handover-procedure/</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>https://pmri.in/epccompletion/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
       <c r="A22" s="3" t="inlineStr"/>
       <c r="B22" s="3" t="inlineStr">
         <is>
@@ -765,12 +852,16 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.pmi.org/learning/library/realizing-engineering-procurement-construction-projects-7173
-2. https://rkstrainings.com/what-is-project-management-in-epc/</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="48" customHeight="1">
+          <t>https://www.pmi.org/learning/library/realizing-engineering-procurement-construction-projects-7173</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>https://rkstrainings.com/what-is-project-management-in-epc/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Project Mobilization and Site Establishment Process</t>
@@ -783,12 +874,16 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>1. https://lauwtjunnji.weebly.com/uploads/1/0/1/7/10171621/fidic_-_conditions_of_contract_for_epc_(turnkey)_projects_(1999).pdf
-2. https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="48" customHeight="1">
+          <t>https://lauwtjunnji.weebly.com/uploads/1/0/1/7/10171621/fidic_-_conditions_of_contract_for_epc_(turnkey)_projects_(1999).pdf</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
       <c r="A24" s="3" t="inlineStr"/>
       <c r="B24" s="3" t="inlineStr">
         <is>
@@ -797,12 +892,16 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.substationfaults.com/electrical-substation-construction/
-2. https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="48" customHeight="1">
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1">
       <c r="A25" s="3" t="inlineStr"/>
       <c r="B25" s="3" t="inlineStr">
         <is>
@@ -811,12 +910,16 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>1. https://prismecs.com/blog/understanding-the-lifecycle-of-epc-solutions-services
-2. https://rkstrainings.com/what-is-project-management-in-epc/</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="48" customHeight="1">
+          <t>https://prismecs.com/blog/understanding-the-lifecycle-of-epc-solutions-services</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>https://rkstrainings.com/what-is-project-management-in-epc/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
       <c r="A26" s="3" t="inlineStr"/>
       <c r="B26" s="3" t="inlineStr">
         <is>
@@ -825,12 +928,16 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning
-2. https://www.substationfaults.com/electrical-substation-construction/</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="40" customHeight="1">
       <c r="A27" s="3" t="inlineStr"/>
       <c r="B27" s="3" t="inlineStr">
         <is>
@@ -839,12 +946,16 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>1. https://electra.cigre.org/311-august-2020/technical-brochures/guidelines-for-safe-work-methods-in-substations.html
-2. https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="48" customHeight="1">
+          <t>https://electra.cigre.org/311-august-2020/technical-brochures/guidelines-for-safe-work-methods-in-substations.html</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="40" customHeight="1">
       <c r="A28" s="3" t="inlineStr"/>
       <c r="B28" s="3" t="inlineStr">
         <is>
@@ -853,12 +964,16 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning
-2. https://www.substationfaults.com/electrical-substation-construction/</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="40" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Survey, Geotechnical Investigation and Design Release Process</t>
@@ -871,12 +986,16 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-design-engineering
-2. https://keentelengineering.com/a-guide-to-the-substation-design-process</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-design-engineering</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>https://keentelengineering.com/a-guide-to-the-substation-design-process</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="40" customHeight="1">
       <c r="A30" s="3" t="inlineStr"/>
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -885,12 +1004,16 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>1. https://keentelengineering.com/a-guide-to-the-substation-design-process
-2. https://www.substationfaults.com/electrical-substation-construction/</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="48" customHeight="1">
+          <t>https://keentelengineering.com/a-guide-to-the-substation-design-process</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="40" customHeight="1">
       <c r="A31" s="3" t="inlineStr"/>
       <c r="B31" s="3" t="inlineStr">
         <is>
@@ -899,12 +1022,16 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-design-engineering
-2. https://keentelengineering.com/a-guide-to-the-substation-design-process</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-design-engineering</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>https://keentelengineering.com/a-guide-to-the-substation-design-process</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="40" customHeight="1">
       <c r="A32" s="3" t="inlineStr"/>
       <c r="B32" s="3" t="inlineStr">
         <is>
@@ -913,12 +1040,16 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>1. https://keentelengineering.com/a-guide-to-the-substation-design-process
-2. https://rkstrainings.com/what-is-project-management-in-epc/</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="48" customHeight="1">
+          <t>https://keentelengineering.com/a-guide-to-the-substation-design-process</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>https://rkstrainings.com/what-is-project-management-in-epc/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="40" customHeight="1">
       <c r="A33" s="3" t="inlineStr"/>
       <c r="B33" s="3" t="inlineStr">
         <is>
@@ -927,12 +1058,16 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/turnkey-substation-technical-documentation
-2. https://www.pmi.org/learning/library/realizing-engineering-procurement-construction-projects-7173</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/turnkey-substation-technical-documentation</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pmi.org/learning/library/realizing-engineering-procurement-construction-projects-7173</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="40" customHeight="1">
       <c r="A34" s="3" t="inlineStr"/>
       <c r="B34" s="3" t="inlineStr">
         <is>
@@ -941,12 +1076,16 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-design-engineering
-2. https://electrical-engineering-portal.com/turnkey-substation-technical-documentation</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-design-engineering</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical-engineering-portal.com/turnkey-substation-technical-documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="40" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Detailed Engineering and IFC Release Process</t>
@@ -959,12 +1098,16 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-design-engineering
-2. https://www.academia.edu/93132452/ElECTRIC_POWER_SUBSTATIONS_ENGINEERING</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-design-engineering</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>https://www.academia.edu/93132452/ElECTRIC_POWER_SUBSTATIONS_ENGINEERING</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="40" customHeight="1">
       <c r="A36" s="3" t="inlineStr"/>
       <c r="B36" s="3" t="inlineStr">
         <is>
@@ -973,12 +1116,16 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-design-engineering
-2. https://keentelengineering.com/ieee-compliant-ehv-hv-mv-substation-design-services-by-keentel-engineering</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-design-engineering</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>https://keentelengineering.com/ieee-compliant-ehv-hv-mv-substation-design-services-by-keentel-engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="40" customHeight="1">
       <c r="A37" s="3" t="inlineStr"/>
       <c r="B37" s="3" t="inlineStr">
         <is>
@@ -987,12 +1134,16 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>1. https://keentelengineering.com/a-guide-to-the-substation-design-process
-2. https://www.academia.edu/93132452/ElECTRIC_POWER_SUBSTATIONS_ENGINEERING</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="48" customHeight="1">
+          <t>https://keentelengineering.com/a-guide-to-the-substation-design-process</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>https://www.academia.edu/93132452/ElECTRIC_POWER_SUBSTATIONS_ENGINEERING</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="40" customHeight="1">
       <c r="A38" s="3" t="inlineStr"/>
       <c r="B38" s="3" t="inlineStr">
         <is>
@@ -1001,12 +1152,16 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-design-engineering
-2. https://keentelengineering.com/a-guide-to-the-substation-design-process</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-design-engineering</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>https://keentelengineering.com/a-guide-to-the-substation-design-process</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="40" customHeight="1">
       <c r="A39" s="3" t="inlineStr"/>
       <c r="B39" s="3" t="inlineStr">
         <is>
@@ -1015,12 +1170,16 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>1. https://seclab.illinois.edu/wp-content/uploads/2011/03/iec61850-intro.pdf
-2. https://library.e.abb.com/public/5ea2620c3dec4376a1540fc2b07a18b7/IEC%2061850%20Overview_Self.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="48" customHeight="1">
+          <t>https://seclab.illinois.edu/wp-content/uploads/2011/03/iec61850-intro.pdf</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>https://library.e.abb.com/public/5ea2620c3dec4376a1540fc2b07a18b7/IEC%2061850%20Overview_Self.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="40" customHeight="1">
       <c r="A40" s="3" t="inlineStr"/>
       <c r="B40" s="3" t="inlineStr">
         <is>
@@ -1029,12 +1188,16 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>1. https://keentelengineering.com/ieee-compliant-ehv-hv-mv-substation-design-services-by-keentel-engineering
-2. https://www.academia.edu/93132452/ElECTRIC_POWER_SUBSTATIONS_ENGINEERING</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="48" customHeight="1">
+          <t>https://keentelengineering.com/ieee-compliant-ehv-hv-mv-substation-design-services-by-keentel-engineering</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>https://www.academia.edu/93132452/ElECTRIC_POWER_SUBSTATIONS_ENGINEERING</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="40" customHeight="1">
       <c r="A41" s="3" t="inlineStr"/>
       <c r="B41" s="3" t="inlineStr">
         <is>
@@ -1043,12 +1206,16 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-design-engineering
-2. https://keentelengineering.com/ieee-compliant-ehv-hv-mv-substation-design-services-by-keentel-engineering</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-design-engineering</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>https://keentelengineering.com/ieee-compliant-ehv-hv-mv-substation-design-services-by-keentel-engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="40" customHeight="1">
       <c r="A42" s="3" t="inlineStr"/>
       <c r="B42" s="3" t="inlineStr">
         <is>
@@ -1057,12 +1224,16 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>1. https://keentelengineering.com/ieee-compliant-ehv-hv-mv-substation-design-services-by-keentel-engineering
-2. https://www.academia.edu/93132452/ElECTRIC_POWER_SUBSTATIONS_ENGINEERING</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="48" customHeight="1">
+          <t>https://keentelengineering.com/ieee-compliant-ehv-hv-mv-substation-design-services-by-keentel-engineering</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>https://www.academia.edu/93132452/ElECTRIC_POWER_SUBSTATIONS_ENGINEERING</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="40" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
           <t>Submit for Approval – Client Submission Process</t>
@@ -1075,12 +1246,16 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/turnkey-substation-technical-documentation
-2. https://keentelengineering.com/a-guide-to-the-substation-design-process</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/turnkey-substation-technical-documentation</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>https://keentelengineering.com/a-guide-to-the-substation-design-process</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="40" customHeight="1">
       <c r="A44" s="3" t="inlineStr"/>
       <c r="B44" s="3" t="inlineStr">
         <is>
@@ -1089,12 +1264,16 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/turnkey-substation-technical-documentation
-2. https://www.pmi.org/learning/library/realizing-engineering-procurement-construction-projects-7173</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/turnkey-substation-technical-documentation</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pmi.org/learning/library/realizing-engineering-procurement-construction-projects-7173</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="40" customHeight="1">
       <c r="A45" s="3" t="inlineStr"/>
       <c r="B45" s="3" t="inlineStr">
         <is>
@@ -1103,12 +1282,16 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/turnkey-substation-technical-documentation
-2. https://rkstrainings.com/what-is-project-management-in-epc/</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/turnkey-substation-technical-documentation</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>https://rkstrainings.com/what-is-project-management-in-epc/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="40" customHeight="1">
       <c r="A46" s="3" t="inlineStr"/>
       <c r="B46" s="3" t="inlineStr">
         <is>
@@ -1117,12 +1300,16 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/turnkey-substation-technical-documentation
-2. https://www.academia.edu/93132452/ElECTRIC_POWER_SUBSTATIONS_ENGINEERING</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/turnkey-substation-technical-documentation</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>https://www.academia.edu/93132452/ElECTRIC_POWER_SUBSTATIONS_ENGINEERING</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="40" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Procurement, Vendor Approval and Manufacturing Process</t>
@@ -1135,12 +1322,16 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>1. https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents
-2. https://rkstrainings.com/what-is-project-management-in-epc/</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="48" customHeight="1">
+          <t>https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>https://rkstrainings.com/what-is-project-management-in-epc/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="40" customHeight="1">
       <c r="A48" s="3" t="inlineStr"/>
       <c r="B48" s="3" t="inlineStr">
         <is>
@@ -1149,12 +1340,16 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>1. https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents
-2. https://electrical-engineering-portal.com/checks-for-successful-substation-factory-acceptance-testing</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="48" customHeight="1">
+          <t>https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical-engineering-portal.com/checks-for-successful-substation-factory-acceptance-testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="40" customHeight="1">
       <c r="A49" s="3" t="inlineStr"/>
       <c r="B49" s="3" t="inlineStr">
         <is>
@@ -1163,12 +1358,16 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>1. https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents
-2. https://www.euci.com/event_post/epc-contracts/</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="48" customHeight="1">
+          <t>https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>https://www.euci.com/event_post/epc-contracts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="40" customHeight="1">
       <c r="A50" s="3" t="inlineStr"/>
       <c r="B50" s="3" t="inlineStr">
         <is>
@@ -1177,12 +1376,16 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>1. https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents
-2. https://keentelengineering.com/substation-testing-lifecycle-fat-vs-sat</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="48" customHeight="1">
+          <t>https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>https://keentelengineering.com/substation-testing-lifecycle-fat-vs-sat</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="40" customHeight="1">
       <c r="A51" s="3" t="inlineStr"/>
       <c r="B51" s="3" t="inlineStr">
         <is>
@@ -1191,12 +1394,16 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>1. https://lauwtjunnji.weebly.com/uploads/1/0/1/7/10171621/fidic_-_conditions_of_contract_for_epc_(turnkey)_projects_(1999).pdf
-2. https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="48" customHeight="1">
+          <t>https://lauwtjunnji.weebly.com/uploads/1/0/1/7/10171621/fidic_-_conditions_of_contract_for_epc_(turnkey)_projects_(1999).pdf</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="40" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Manufacturing Execution, FAT Testing and Dispatch Process</t>
@@ -1209,12 +1416,16 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/checks-for-successful-substation-factory-acceptance-testing
-2. https://keentelengineering.com/substation-testing-lifecycle-fat-vs-sat</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/checks-for-successful-substation-factory-acceptance-testing</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>https://keentelengineering.com/substation-testing-lifecycle-fat-vs-sat</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="40" customHeight="1">
       <c r="A53" s="3" t="inlineStr"/>
       <c r="B53" s="3" t="inlineStr">
         <is>
@@ -1223,12 +1434,16 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/substation-equipment-type-testing-factory-site-acceptance-testing-fat-sat
-2. https://electrical-engineering-portal.com/transformer-factory-acceptance-tests-final-inspections</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/substation-equipment-type-testing-factory-site-acceptance-testing-fat-sat</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical-engineering-portal.com/transformer-factory-acceptance-tests-final-inspections</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="40" customHeight="1">
       <c r="A54" s="3" t="inlineStr"/>
       <c r="B54" s="3" t="inlineStr">
         <is>
@@ -1237,12 +1452,16 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/substation-equipment-type-testing-factory-site-acceptance-testing-fat-sat
-2. https://keentelengineering.com/substation-testing-lifecycle-fat-vs-sat</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/substation-equipment-type-testing-factory-site-acceptance-testing-fat-sat</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>https://keentelengineering.com/substation-testing-lifecycle-fat-vs-sat</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="40" customHeight="1">
       <c r="A55" s="3" t="inlineStr"/>
       <c r="B55" s="3" t="inlineStr">
         <is>
@@ -1251,12 +1470,16 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/checks-for-successful-substation-factory-acceptance-testing
-2. https://electrical-engineering-portal.com/res3/FAT-SAT-OF-electrical-and-automation-systems.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/checks-for-successful-substation-factory-acceptance-testing</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical-engineering-portal.com/res3/FAT-SAT-OF-electrical-and-automation-systems.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="40" customHeight="1">
       <c r="A56" s="3" t="inlineStr"/>
       <c r="B56" s="3" t="inlineStr">
         <is>
@@ -1265,12 +1488,16 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>1. https://keentelengineering.com/substation-testing-lifecycle-fat-vs-sat
-2. https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="48" customHeight="1">
+          <t>https://keentelengineering.com/substation-testing-lifecycle-fat-vs-sat</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="40" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
           <t>Logistics, Transportation and Material Receipt Process</t>
@@ -1283,12 +1510,16 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>1. https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents
-2. https://rkstrainings.com/what-is-project-management-in-epc/</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="48" customHeight="1">
+          <t>https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>https://rkstrainings.com/what-is-project-management-in-epc/</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="40" customHeight="1">
       <c r="A58" s="3" t="inlineStr"/>
       <c r="B58" s="3" t="inlineStr">
         <is>
@@ -1297,12 +1528,16 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>1. https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents
-2. https://keentelengineering.com/substation-testing-lifecycle-fat-vs-sat</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="48" customHeight="1">
+          <t>https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>https://keentelengineering.com/substation-testing-lifecycle-fat-vs-sat</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="40" customHeight="1">
       <c r="A59" s="3" t="inlineStr"/>
       <c r="B59" s="3" t="inlineStr">
         <is>
@@ -1311,12 +1546,16 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>1. https://rkstrainings.com/what-is-project-management-in-epc/
-2. https://prismecs.com/blog/understanding-the-lifecycle-of-epc-solutions-services</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="48" customHeight="1">
+          <t>https://rkstrainings.com/what-is-project-management-in-epc/</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>https://prismecs.com/blog/understanding-the-lifecycle-of-epc-solutions-services</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="40" customHeight="1">
       <c r="A60" s="3" t="inlineStr"/>
       <c r="B60" s="3" t="inlineStr">
         <is>
@@ -1325,12 +1564,16 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.substationfaults.com/electrical-substation-construction/
-2. https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="48" customHeight="1">
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="40" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
           <t>Material Receipt, Inspection and Installation Release Process</t>
@@ -1343,12 +1586,16 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.substationfaults.com/electrical-substation-construction/
-2. https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="48" customHeight="1">
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="40" customHeight="1">
       <c r="A62" s="3" t="inlineStr"/>
       <c r="B62" s="3" t="inlineStr">
         <is>
@@ -1357,12 +1604,16 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>1. https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents
-2. https://www.substationfaults.com/electrical-substation-construction/</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="48" customHeight="1">
+          <t>https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="40" customHeight="1">
       <c r="A63" s="3" t="inlineStr"/>
       <c r="B63" s="3" t="inlineStr">
         <is>
@@ -1371,12 +1622,16 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/substation-equipment-type-testing-factory-site-acceptance-testing-fat-sat
-2. https://keentelengineering.com/substation-testing-lifecycle-fat-vs-sat</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/substation-equipment-type-testing-factory-site-acceptance-testing-fat-sat</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>https://keentelengineering.com/substation-testing-lifecycle-fat-vs-sat</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="40" customHeight="1">
       <c r="A64" s="3" t="inlineStr"/>
       <c r="B64" s="3" t="inlineStr">
         <is>
@@ -1385,12 +1640,16 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>1. https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents
-2. https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="48" customHeight="1">
+          <t>https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="40" customHeight="1">
       <c r="A65" s="3" t="inlineStr"/>
       <c r="B65" s="3" t="inlineStr">
         <is>
@@ -1399,12 +1658,16 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>1. https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents
-2. https://rkstrainings.com/what-is-project-management-in-epc/</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="48" customHeight="1">
+          <t>https://blog.projectmaterials.com/category/epc-projects/procurement-logistics/project-procurement-documents</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>https://rkstrainings.com/what-is-project-management-in-epc/</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="40" customHeight="1">
       <c r="A66" s="3" t="inlineStr"/>
       <c r="B66" s="3" t="inlineStr">
         <is>
@@ -1413,12 +1676,16 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning
-2. https://www.substationfaults.com/electrical-substation-construction/</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="40" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
           <t>Civil Construction and Structural Readiness Process</t>
@@ -1431,12 +1698,16 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.substationfaults.com/electrical-substation-construction/
-2. https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="48" customHeight="1">
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="40" customHeight="1">
       <c r="A68" s="3" t="inlineStr"/>
       <c r="B68" s="3" t="inlineStr">
         <is>
@@ -1445,12 +1716,16 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.substationfaults.com/electrical-substation-construction/
-2. https://electra.cigre.org/311-august-2020/technical-brochures/guidelines-for-safe-work-methods-in-substations.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="48" customHeight="1">
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>https://electra.cigre.org/311-august-2020/technical-brochures/guidelines-for-safe-work-methods-in-substations.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="40" customHeight="1">
       <c r="A69" s="3" t="inlineStr"/>
       <c r="B69" s="3" t="inlineStr">
         <is>
@@ -1459,12 +1734,16 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning
-2. https://www.substationfaults.com/electrical-substation-construction/</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="40" customHeight="1">
       <c r="A70" s="3" t="inlineStr"/>
       <c r="B70" s="3" t="inlineStr">
         <is>
@@ -1473,12 +1752,16 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning
-2. https://electra.cigre.org/311-august-2020/technical-brochures/guidelines-for-safe-work-methods-in-substations.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>https://electra.cigre.org/311-august-2020/technical-brochures/guidelines-for-safe-work-methods-in-substations.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="40" customHeight="1">
       <c r="A71" s="3" t="inlineStr"/>
       <c r="B71" s="3" t="inlineStr">
         <is>
@@ -1487,12 +1770,16 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.substationfaults.com/electrical-substation-construction/
-2. https://electra.cigre.org/311-august-2020/technical-brochures/guidelines-for-safe-work-methods-in-substations.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="48" customHeight="1">
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>https://electra.cigre.org/311-august-2020/technical-brochures/guidelines-for-safe-work-methods-in-substations.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="40" customHeight="1">
       <c r="A72" s="3" t="inlineStr"/>
       <c r="B72" s="3" t="inlineStr">
         <is>
@@ -1501,12 +1788,16 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/
-2. https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="40" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
           <t>Equipment Erection, Mechanical Installation and Cabling Readiness Process</t>
@@ -1519,12 +1810,16 @@
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning
-2. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="40" customHeight="1">
       <c r="A74" s="3" t="inlineStr"/>
       <c r="B74" s="3" t="inlineStr">
         <is>
@@ -1533,12 +1828,16 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning
-2. https://electra.cigre.org/311-august-2020/technical-brochures/guidelines-for-safe-work-methods-in-substations.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>https://electra.cigre.org/311-august-2020/technical-brochures/guidelines-for-safe-work-methods-in-substations.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="40" customHeight="1">
       <c r="A75" s="3" t="inlineStr"/>
       <c r="B75" s="3" t="inlineStr">
         <is>
@@ -1547,12 +1846,16 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/transformer-factory-acceptance-tests-final-inspections
-2. https://www.substationfaults.com/electrical-substation-construction/</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/transformer-factory-acceptance-tests-final-inspections</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="40" customHeight="1">
       <c r="A76" s="3" t="inlineStr"/>
       <c r="B76" s="3" t="inlineStr">
         <is>
@@ -1561,12 +1864,16 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>1. https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning
-2. https://keentelengineering.com/ieee-compliant-ehv-hv-mv-substation-design-services-by-keentel-engineering</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="48" customHeight="1">
+          <t>https://electrical-engineering-portal.com/power-substation-project-design-construction-erection-commissioning</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>https://keentelengineering.com/ieee-compliant-ehv-hv-mv-substation-design-services-by-keentel-engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="40" customHeight="1">
       <c r="A77" s="3" t="inlineStr"/>
       <c r="B77" s="3" t="inlineStr">
         <is>
@@ -1575,12 +1882,16 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/
-2. https://powersynchro.com/substation-commissioning-checklist/</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>https://powersynchro.com/substation-commissioning-checklist/</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="40" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
           <t>Cabling, Termination, Testing and SAS Readiness Process</t>
@@ -1593,12 +1904,16 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.substationfaults.com/electrical-substation-construction/
-2. https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="48" customHeight="1">
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="40" customHeight="1">
       <c r="A79" s="3" t="inlineStr"/>
       <c r="B79" s="3" t="inlineStr">
         <is>
@@ -1607,12 +1922,16 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.substationfaults.com/electrical-substation-construction/
-2. https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="48" customHeight="1">
+          <t>https://www.substationfaults.com/electrical-substation-construction/</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="40" customHeight="1">
       <c r="A80" s="3" t="inlineStr"/>
       <c r="B80" s="3" t="inlineStr">
         <is>
@@ -1621,12 +1940,16 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/
-2. https://powersynchro.com/substation-commissioning-checklist/</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>https://powersynchro.com/substation-commissioning-checklist/</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="40" customHeight="1">
       <c r="A81" s="3" t="inlineStr"/>
       <c r="B81" s="3" t="inlineStr">
         <is>
@@ -1635,12 +1958,16 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>1. https://instrumentationtools.com/scada-for-substation-automation/
-2. https://seclab.illinois.edu/wp-content/uploads/2011/03/iec61850-intro.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="48" customHeight="1">
+          <t>https://instrumentationtools.com/scada-for-substation-automation/</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>https://seclab.illinois.edu/wp-content/uploads/2011/03/iec61850-intro.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="40" customHeight="1">
       <c r="A82" s="3" t="inlineStr"/>
       <c r="B82" s="3" t="inlineStr">
         <is>
@@ -1649,12 +1976,16 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-4-scada-and-comms-systems
-2. https://powersynchro.com/substation-commissioning-checklist/</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-4-scada-and-comms-systems</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>https://powersynchro.com/substation-commissioning-checklist/</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="40" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
           <t>SAS / SCADA Integration, Functional Testing and Pre-Commissioning Readiness Process</t>
@@ -1667,12 +1998,16 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>1. https://seclab.illinois.edu/wp-content/uploads/2011/03/iec61850-intro.pdf
-2. https://library.e.abb.com/public/5ea2620c3dec4376a1540fc2b07a18b7/IEC%2061850%20Overview_Self.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="48" customHeight="1">
+          <t>https://seclab.illinois.edu/wp-content/uploads/2011/03/iec61850-intro.pdf</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>https://library.e.abb.com/public/5ea2620c3dec4376a1540fc2b07a18b7/IEC%2061850%20Overview_Self.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="40" customHeight="1">
       <c r="A84" s="3" t="inlineStr"/>
       <c r="B84" s="3" t="inlineStr">
         <is>
@@ -1681,12 +2016,16 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-4-scada-and-comms-systems
-2. https://instrumentationtools.com/scada-for-substation-automation/</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-4-scada-and-comms-systems</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>https://instrumentationtools.com/scada-for-substation-automation/</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="40" customHeight="1">
       <c r="A85" s="3" t="inlineStr"/>
       <c r="B85" s="3" t="inlineStr">
         <is>
@@ -1695,12 +2034,16 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/
-2. https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="40" customHeight="1">
       <c r="A86" s="3" t="inlineStr"/>
       <c r="B86" s="3" t="inlineStr">
         <is>
@@ -1709,12 +2052,16 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-4-scada-and-comms-systems
-2. https://mbcontrol.com/understanding-substation-automation-systems/</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-4-scada-and-comms-systems</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>https://mbcontrol.com/understanding-substation-automation-systems/</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="40" customHeight="1">
       <c r="A87" s="3" t="inlineStr"/>
       <c r="B87" s="3" t="inlineStr">
         <is>
@@ -1723,12 +2070,16 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>1. https://powersynchro.com/substation-commissioning-checklist/
-2. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="48" customHeight="1">
+          <t>https://powersynchro.com/substation-commissioning-checklist/</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="40" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
           <t>Pre-Commissioning Testing, System Validation and Commissioning Readiness Process</t>
@@ -1741,12 +2092,16 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/
-2. https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="40" customHeight="1">
       <c r="A89" s="3" t="inlineStr"/>
       <c r="B89" s="3" t="inlineStr">
         <is>
@@ -1755,12 +2110,16 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/
-2. https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="40" customHeight="1">
       <c r="A90" s="3" t="inlineStr"/>
       <c r="B90" s="3" t="inlineStr">
         <is>
@@ -1769,12 +2128,16 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/
-2. https://elliotengineeringinc.com/testing-and-commissioning/</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>https://elliotengineeringinc.com/testing-and-commissioning/</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="40" customHeight="1">
       <c r="A91" s="3" t="inlineStr"/>
       <c r="B91" s="3" t="inlineStr">
         <is>
@@ -1783,12 +2146,16 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/
-2. https://powersynchro.com/substation-commissioning-checklist/</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>https://powersynchro.com/substation-commissioning-checklist/</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="40" customHeight="1">
       <c r="A92" s="3" t="inlineStr"/>
       <c r="B92" s="3" t="inlineStr">
         <is>
@@ -1797,12 +2164,16 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/
-2. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="40" customHeight="1">
       <c r="A93" s="3" t="inlineStr"/>
       <c r="B93" s="3" t="inlineStr">
         <is>
@@ -1811,12 +2182,16 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/
-2. https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-2-pre-commissioning-inspections/</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="40" customHeight="1">
       <c r="A94" s="3" t="inlineStr"/>
       <c r="B94" s="3" t="inlineStr">
         <is>
@@ -1825,12 +2200,16 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>1. https://powersynchro.com/substation-commissioning-checklist/
-2. https://pmri.in/epccompletion/</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="48" customHeight="1">
+          <t>https://powersynchro.com/substation-commissioning-checklist/</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>https://pmri.in/epccompletion/</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="40" customHeight="1">
       <c r="A95" s="3" t="inlineStr"/>
       <c r="B95" s="3" t="inlineStr">
         <is>
@@ -1839,12 +2218,16 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/
-2. https://powersynchro.com/substation-commissioning-checklist/</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>https://powersynchro.com/substation-commissioning-checklist/</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="40" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
           <t>Final Commissioning, Initial Charging and Energization Readiness Process</t>
@@ -1857,12 +2240,16 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/
-2. https://powersynchro.com/substation-commissioning-checklist/</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>https://powersynchro.com/substation-commissioning-checklist/</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="40" customHeight="1">
       <c r="A97" s="3" t="inlineStr"/>
       <c r="B97" s="3" t="inlineStr">
         <is>
@@ -1871,12 +2258,16 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/
-2. https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="40" customHeight="1">
       <c r="A98" s="3" t="inlineStr"/>
       <c r="B98" s="3" t="inlineStr">
         <is>
@@ -1885,12 +2276,16 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/
-2. https://powersynchro.com/substation-commissioning-checklist/</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>https://powersynchro.com/substation-commissioning-checklist/</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="40" customHeight="1">
       <c r="A99" s="3" t="inlineStr"/>
       <c r="B99" s="3" t="inlineStr">
         <is>
@@ -1899,12 +2294,16 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/
-2. https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="40" customHeight="1">
       <c r="A100" s="3" t="inlineStr"/>
       <c r="B100" s="3" t="inlineStr">
         <is>
@@ -1913,12 +2312,16 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/
-2. https://elliotengineeringinc.com/testing-and-commissioning/</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>https://elliotengineeringinc.com/testing-and-commissioning/</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="40" customHeight="1">
       <c r="A101" s="3" t="inlineStr"/>
       <c r="B101" s="3" t="inlineStr">
         <is>
@@ -1927,12 +2330,16 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/
-2. https://powersynchro.com/substation-commissioning-checklist/</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>https://powersynchro.com/substation-commissioning-checklist/</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="40" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
         <is>
           <t>Final Energization and Grid Synchronization Process</t>
@@ -1945,12 +2352,16 @@
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/
-2. https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="40" customHeight="1">
       <c r="A103" s="3" t="inlineStr"/>
       <c r="B103" s="3" t="inlineStr">
         <is>
@@ -1959,12 +2370,16 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/
-2. https://powersynchro.com/substation-commissioning-checklist/</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>https://powersynchro.com/substation-commissioning-checklist/</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="40" customHeight="1">
       <c r="A104" s="3" t="inlineStr"/>
       <c r="B104" s="3" t="inlineStr">
         <is>
@@ -1973,12 +2388,16 @@
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/
-2. https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="40" customHeight="1">
       <c r="A105" s="3" t="inlineStr"/>
       <c r="B105" s="3" t="inlineStr">
         <is>
@@ -1987,12 +2406,16 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/
-2. https://powersynchro.com/substation-commissioning-checklist/</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testing-part-3-field-testing/</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>https://powersynchro.com/substation-commissioning-checklist/</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="40" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
           <t>Trial Run and Performance Stabilization Process</t>
@@ -2005,12 +2428,16 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/
-2. https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>https://electrical4learning.blogspot.com/2024/11/method-statement-for-testing-and-commissioning-of-substation-equipments.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="40" customHeight="1">
       <c r="A107" s="3" t="inlineStr"/>
       <c r="B107" s="3" t="inlineStr">
         <is>
@@ -2019,12 +2446,16 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.ncbi.nlm.nih.gov/pmc/articles/PMC12431182/
-2. https://instrumentationtools.com/scada-for-substation-automation/</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="48" customHeight="1">
+          <t>https://www.ncbi.nlm.nih.gov/pmc/articles/PMC12431182/</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>https://instrumentationtools.com/scada-for-substation-automation/</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="40" customHeight="1">
       <c r="A108" s="3" t="inlineStr"/>
       <c r="B108" s="3" t="inlineStr">
         <is>
@@ -2033,12 +2464,16 @@
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>1. https://relgrow.com/resources/dlp-full-form-in-construction/
-2. https://www.mastt.com/blogs/defects-liability-period</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="48" customHeight="1">
+          <t>https://relgrow.com/resources/dlp-full-form-in-construction/</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mastt.com/blogs/defects-liability-period</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="40" customHeight="1">
       <c r="A109" s="3" t="inlineStr"/>
       <c r="B109" s="3" t="inlineStr">
         <is>
@@ -2047,12 +2482,16 @@
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>1. https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/
-2. https://pmri.in/epccompletion/</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="48" customHeight="1">
+          <t>https://eepower.com/technical-articles/substation-commissioning-and-testingpart-1-scope-and-workflow/</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>https://pmri.in/epccompletion/</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="40" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
         <is>
           <t>Project Closure, Client Acceptance and Final Handover Process</t>
@@ -2065,12 +2504,16 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>1. https://pmri.in/epccompletion/
-2. https://projectmanagement123.com/project-completion-and-handover-procedure/</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="48" customHeight="1">
+          <t>https://pmri.in/epccompletion/</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>https://projectmanagement123.com/project-completion-and-handover-procedure/</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="40" customHeight="1">
       <c r="A111" s="3" t="inlineStr"/>
       <c r="B111" s="3" t="inlineStr">
         <is>
@@ -2079,12 +2522,16 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>1. https://pmri.in/epccompletion/
-2. https://projectmanagement123.com/project-completion-and-handover-procedure/</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="48" customHeight="1">
+          <t>https://pmri.in/epccompletion/</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>https://projectmanagement123.com/project-completion-and-handover-procedure/</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="40" customHeight="1">
       <c r="A112" s="3" t="inlineStr"/>
       <c r="B112" s="3" t="inlineStr">
         <is>
@@ -2093,12 +2540,16 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>1. https://projectmanagement123.com/project-completion-and-handover-procedure/
-2. https://pmri.in/epccompletion/</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="48" customHeight="1">
+          <t>https://projectmanagement123.com/project-completion-and-handover-procedure/</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>https://pmri.in/epccompletion/</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="40" customHeight="1">
       <c r="A113" s="3" t="inlineStr"/>
       <c r="B113" s="3" t="inlineStr">
         <is>
@@ -2107,12 +2558,16 @@
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>1. https://relgrow.com/resources/dlp-full-form-in-construction/
-2. https://www.mastt.com/blogs/defects-liability-period</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="48" customHeight="1">
+          <t>https://relgrow.com/resources/dlp-full-form-in-construction/</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mastt.com/blogs/defects-liability-period</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="40" customHeight="1">
       <c r="A114" s="3" t="inlineStr"/>
       <c r="B114" s="3" t="inlineStr">
         <is>
@@ -2121,12 +2576,16 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>1. https://projectmanagement123.com/project-completion-and-handover-procedure/
-2. https://pmri.in/epccompletion/</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="48" customHeight="1">
+          <t>https://projectmanagement123.com/project-completion-and-handover-procedure/</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>https://pmri.in/epccompletion/</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="40" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
         <is>
           <t>Defect Liability Period (DLP), Warranty Support and Final Acceptance Process</t>
@@ -2139,12 +2598,16 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.mastt.com/blogs/defects-liability-period
-2. https://relgrow.com/resources/dlp-full-form-in-construction/</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="48" customHeight="1">
+          <t>https://www.mastt.com/blogs/defects-liability-period</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>https://relgrow.com/resources/dlp-full-form-in-construction/</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="40" customHeight="1">
       <c r="A116" s="3" t="inlineStr"/>
       <c r="B116" s="3" t="inlineStr">
         <is>
@@ -2153,12 +2616,16 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.mastt.com/blogs/defects-liability-period
-2. https://www.turtons.com/blog/what-is-the-defects-liability-period</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" ht="48" customHeight="1">
+          <t>https://www.mastt.com/blogs/defects-liability-period</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>https://www.turtons.com/blog/what-is-the-defects-liability-period</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="40" customHeight="1">
       <c r="A117" s="3" t="inlineStr"/>
       <c r="B117" s="3" t="inlineStr">
         <is>
@@ -2167,12 +2634,16 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>1. https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/
-2. https://www.mastt.com/blogs/defects-liability-period</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" ht="48" customHeight="1">
+          <t>https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mastt.com/blogs/defects-liability-period</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="40" customHeight="1">
       <c r="A118" s="3" t="inlineStr"/>
       <c r="B118" s="3" t="inlineStr">
         <is>
@@ -2181,12 +2652,16 @@
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>1. https://www.mastt.com/blogs/defects-liability-period
-2. https://lauwtjunnji.weebly.com/uploads/1/0/1/7/10171621/fidic_-_conditions_of_contract_for_epc_(turnkey)_projects_(1999).pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="119" ht="48" customHeight="1">
+          <t>https://www.mastt.com/blogs/defects-liability-period</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>https://lauwtjunnji.weebly.com/uploads/1/0/1/7/10171621/fidic_-_conditions_of_contract_for_epc_(turnkey)_projects_(1999).pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="40" customHeight="1">
       <c r="A119" s="2" t="inlineStr">
         <is>
           <t>Final Acceptance Certificate (FAC), Contract Closure and Project Closeout Process</t>
@@ -2199,12 +2674,16 @@
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>1. https://relgrow.com/resources/dlp-full-form-in-construction/
-2. https://pmri.in/epccompletion/</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" ht="48" customHeight="1">
+          <t>https://relgrow.com/resources/dlp-full-form-in-construction/</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>https://pmri.in/epccompletion/</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="40" customHeight="1">
       <c r="A120" s="3" t="inlineStr"/>
       <c r="B120" s="3" t="inlineStr">
         <is>
@@ -2213,12 +2692,16 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>1. https://relgrow.com/resources/dlp-full-form-in-construction/
-2. https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/</t>
-        </is>
-      </c>
-    </row>
-    <row r="121" ht="48" customHeight="1">
+          <t>https://relgrow.com/resources/dlp-full-form-in-construction/</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="40" customHeight="1">
       <c r="A121" s="3" t="inlineStr"/>
       <c r="B121" s="3" t="inlineStr">
         <is>
@@ -2227,12 +2710,16 @@
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>1. https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/
-2. https://lauwtjunnji.weebly.com/uploads/1/0/1/7/10171621/fidic_-_conditions_of_contract_for_epc_(turnkey)_projects_(1999).pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="48" customHeight="1">
+          <t>https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>https://lauwtjunnji.weebly.com/uploads/1/0/1/7/10171621/fidic_-_conditions_of_contract_for_epc_(turnkey)_projects_(1999).pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="40" customHeight="1">
       <c r="A122" s="3" t="inlineStr"/>
       <c r="B122" s="3" t="inlineStr">
         <is>
@@ -2241,12 +2728,16 @@
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>1. https://projectmanagement123.com/project-completion-and-handover-procedure/
-2. https://www.pmi.org/learning/library/realizing-engineering-procurement-construction-projects-7173</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" ht="48" customHeight="1">
+          <t>https://projectmanagement123.com/project-completion-and-handover-procedure/</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pmi.org/learning/library/realizing-engineering-procurement-construction-projects-7173</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="40" customHeight="1">
       <c r="A123" s="3" t="inlineStr"/>
       <c r="B123" s="3" t="inlineStr">
         <is>
@@ -2255,13 +2746,263 @@
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>1. https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/
-2. https://www.mastt.com/blogs/defects-liability-period</t>
+          <t>https://constructionlawmadeeasy.com/construction-law/chapter-10/defects-liability-period/</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mastt.com/blogs/defects-liability-period</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C123"/>
+  <autoFilter ref="A1:D123"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId244"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>